<commit_message>
Mark Siu et al. (2026) as in press at Communications Biology
Adds a status column to the papers sheet (build_publications.py already
reads it) so the citation renders as 'Communications Biology: In press'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PEyo4fcfYPxm69SofvuPp6
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="24720" yWindow="9020" windowWidth="57000" windowHeight="23480" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="papers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chapters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dissertations" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="talks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courses" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="posters" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="papers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="chapters" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="dissertations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="talks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="courses" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="posters" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -590,6 +590,11 @@
           <t>data_link</t>
         </is>
       </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="68" customHeight="1">
       <c r="A2" t="inlineStr">
@@ -667,16 +672,12 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>bioRxiv</t>
+          <t>Communications Biology</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>10.64898/2026.04.30.722005v1</t>
-        </is>
-      </c>
+      <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>https://www.biorxiv.org/content/10.64898/2026.04.30.722005v1</t>
@@ -690,6 +691,11 @@
       <c r="L3" s="3" t="inlineStr">
         <is>
           <t>https://db.humanconnectome.org</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>In press</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
List Naturalistic data analysis only as a publication; Clustrix is sole-authored
Removes it from the website's course materials and the CV's open courses,
so it appears once, in the publication lists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PEyo4fcfYPxm69SofvuPp6
</commit_message>
<xml_diff>
--- a/data/publications.xlsx
+++ b/data/publications.xlsx
@@ -3973,7 +3973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -4067,192 +4067,166 @@
     <row r="4" ht="51" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>naturalistic-data.png</t>
+          <t>programming-psych.png</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Naturalistic Data Analysis</t>
+          <t>Introduction to Programming for Psychological Scientists</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>https://naturalistic-data.org/content/intro.html</t>
+          <t>https://github.com/ContextLab/cs-for-psych</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>An online book that includes a collection of state-of-the-art approaches to analyzing naturalistic data.</t>
+          <t>A self-directed open course intended to introduce students to fundamental computational tools used by modern psychological researchers.</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/naturalistic-data-analysis/naturalistic_data_analysis</t>
+          <t>https://github.com/ContextLab/cs-for-psych</t>
         </is>
       </c>
     </row>
     <row r="5" ht="68" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>programming-psych.png</t>
+          <t>lab-tutorials.png</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Introduction to Programming for Psychological Scientists</t>
+          <t>Lab tutorials</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/cs-for-psych</t>
+          <t>https://github.com/ContextLab/CDL-tutorials</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>A self-directed open course intended to introduce students to fundamental computational tools used by modern psychological researchers.</t>
+          <t>A collection of lab tutorials on a range of quantitative and computational topics.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/cs-for-psych</t>
+          <t>https://github.com/ContextLab/CDL-tutorials</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>lab-tutorials.png</t>
+          <t>mind-summer.png</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Lab tutorials</t>
+          <t>Methods in Neuroscience at Dartmouth (MIND)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/CDL-tutorials</t>
+          <t>http://mindsummerschool.org/</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>A collection of lab tutorials on a range of quantitative and computational topics.</t>
+          <t>A 10-day intensive summer course on cutting-edge computational methods.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/CDL-tutorials</t>
+          <t>https://github.com/Summer-MIND</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>mind-summer.png</t>
+          <t>StorytellingWithData-23.webp</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Methods in Neuroscience at Dartmouth (MIND)</t>
+          <t>Storytelling with Data</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>http://mindsummerschool.org/</t>
+          <t>https://github.com/ContextLab/storytelling-with-data</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>A 10-day intensive summer course on cutting-edge computational methods.</t>
+          <t>Data science course aimed at a general audience (no pre-requisites).</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/Summer-MIND</t>
+          <t>https://github.com/ContextLab/storytelling-with-data</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>StorytellingWithData-23.webp</t>
+          <t>MechanicalBrain_Edited.webp</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Storytelling with Data</t>
+          <t>Computational Neuroscience</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/storytelling-with-data</t>
+          <t>https://github.com/ContextLab/computational-neuroscience</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Data science course aimed at a general audience (no pre-requisites).</t>
+          <t>A short University of Pennsylvania summer course that provides an introduction to programming in MATLAB, single-neuron models, ion channel models, basic neural networks, and neural decoding.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>https://github.com/ContextLab/storytelling-with-data</t>
+          <t>https://github.com/ContextLab/computational-neuroscience</t>
         </is>
       </c>
     </row>
     <row r="9" ht="85" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>MechanicalBrain_Edited.webp</t>
+          <t>llm_course.jpg</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Computational Neuroscience</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/computational-neuroscience</t>
+          <t>Models of Language and Communication</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://context-lab.com/llm-course</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>A short University of Pennsylvania summer course that provides an introduction to programming in MATLAB, single-neuron models, ion channel models, basic neural networks, and neural decoding.</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>https://github.com/ContextLab/computational-neuroscience</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>llm_course.jpg</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Models of Language and Communication</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>https://context-lab.com/llm-course</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
           <t>An open course on language models, chatbots, and natural language processing</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>https://github.com/ContextLab/llm-course</t>
         </is>
       </c>
     </row>
+    <row r="10" ht="17" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>